<commit_message>
chore: sync final vendor excel test cases
</commit_message>
<xml_diff>
--- a/swarajya-create/vendor-management/test_data/Create-Vendor-Management.xlsx
+++ b/swarajya-create/vendor-management/test_data/Create-Vendor-Management.xlsx
@@ -784,12 +784,12 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J5" s="0" t="inlineStr">
         <is>
           <t>AUT_VENDOR_POS_06</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="K5" s="0" t="inlineStr">
         <is>
           <t>2026-08-29 20:36:59 | Cancel/Reset button failed to respond</t>
         </is>
@@ -832,7 +832,7 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>To Be Automated</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -842,7 +842,17 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>AUT_VENDOR_POS_07</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-29 20:38:07 | Locator.wait_for: Timeout 8000ms exceeded. Call log:   - waiting for locator("button:has-text('Save'), button:has-text('Submit'), button[type='submit'], button.btn-save").first to be visible </t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(vendor): align locators and routes with staging, achieve 100% test pass rate
</commit_message>
<xml_diff>
--- a/swarajya-create/vendor-management/test_data/Create-Vendor-Management.xlsx
+++ b/swarajya-create/vendor-management/test_data/Create-Vendor-Management.xlsx
@@ -607,7 +607,7 @@
       </c>
       <c r="K2" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 20:34:27</t>
+          <t>2026-08-29 21:02:58</t>
         </is>
       </c>
     </row>
@@ -660,7 +660,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J3" s="0" t="inlineStr">
@@ -670,7 +670,7 @@
       </c>
       <c r="K3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-29 20:35:33 | Locator.wait_for: Timeout 8000ms exceeded. Call log:   - waiting for locator("button:has-text('Save'), button:has-text('Submit'), button[type='submit'], button.btn-save").first to be visible </t>
+          <t>2026-08-29 21:03:10</t>
         </is>
       </c>
     </row>
@@ -717,7 +717,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J4" s="0" t="inlineStr">
@@ -727,7 +727,7 @@
       </c>
       <c r="K4" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 20:35:59 | Vendor 'Acme Corp' not found in vendor management list</t>
+          <t>2026-08-29 21:03:18</t>
         </is>
       </c>
     </row>
@@ -781,7 +781,7 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J5" s="0" t="inlineStr">
@@ -791,7 +791,7 @@
       </c>
       <c r="K5" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 20:36:59 | Cancel/Reset button failed to respond</t>
+          <t>2026-08-29 21:03:22</t>
         </is>
       </c>
     </row>
@@ -842,17 +842,17 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J6" s="0" t="inlineStr">
         <is>
           <t>AUT_VENDOR_POS_07</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-08-29 20:38:07 | Locator.wait_for: Timeout 8000ms exceeded. Call log:   - waiting for locator("button:has-text('Save'), button:has-text('Submit'), button[type='submit'], button.btn-save").first to be visible </t>
+      <c r="K6" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-29 21:03:33</t>
         </is>
       </c>
     </row>
@@ -897,7 +897,7 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>To Be Automated</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
@@ -907,7 +907,17 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J7" s="0" t="inlineStr">
+        <is>
+          <t>AUT_VENDOR_POS_08</t>
+        </is>
+      </c>
+      <c r="K7" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-29 21:03:44</t>
         </is>
       </c>
     </row>
@@ -948,7 +958,7 @@
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>To Be Automated</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
@@ -958,7 +968,17 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J8" s="0" t="inlineStr">
+        <is>
+          <t>AUT_VENDOR_POS_09</t>
+        </is>
+      </c>
+      <c r="K8" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-29 21:03:49</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1021,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>To Be Automated</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -1011,7 +1031,17 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J9" s="0" t="inlineStr">
+        <is>
+          <t>AUT_VENDOR_POS_10</t>
+        </is>
+      </c>
+      <c r="K9" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-29 21:03:59</t>
         </is>
       </c>
     </row>
@@ -1054,7 +1084,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>To Be Automated</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -1064,7 +1094,17 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J10" s="0" t="inlineStr">
+        <is>
+          <t>AUT_VENDOR_POS_11</t>
+        </is>
+      </c>
+      <c r="K10" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-29 21:04:10</t>
         </is>
       </c>
     </row>
@@ -12174,7 +12214,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J2" s="0" t="inlineStr">
@@ -12184,7 +12224,7 @@
       </c>
       <c r="K2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-29 20:19:51 | Locator.wait_for: Timeout 8000ms exceeded. Call log:   - waiting for locator("button:has-text('Save'), button:has-text('Submit'), button[type='submit'], button.btn-save").first to be visible </t>
+          <t>2026-08-29 21:04:34</t>
         </is>
       </c>
     </row>
@@ -12236,7 +12276,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J3" s="0" t="inlineStr">
@@ -12246,7 +12286,7 @@
       </c>
       <c r="K3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-29 20:20:58 | Locator.wait_for: Timeout 8000ms exceeded. Call log:   - waiting for locator("button:has-text('Save'), button:has-text('Submit'), button[type='submit'], button.btn-save").first to be visible </t>
+          <t>2026-08-29 21:04:47</t>
         </is>
       </c>
     </row>
@@ -12298,7 +12338,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J4" s="0" t="inlineStr">
@@ -12308,7 +12348,7 @@
       </c>
       <c r="K4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-29 20:22:07 | Locator.wait_for: Timeout 8000ms exceeded. Call log:   - waiting for locator("button:has-text('Save'), button:has-text('Submit'), button[type='submit'], button.btn-save").first to be visible </t>
+          <t>2026-08-29 21:05:00</t>
         </is>
       </c>
     </row>
@@ -12358,7 +12398,7 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J5" s="0" t="inlineStr">
@@ -12368,7 +12408,7 @@
       </c>
       <c r="K5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-29 20:23:14 | Locator.wait_for: Timeout 8000ms exceeded. Call log:   - waiting for locator("button:has-text('Save'), button:has-text('Submit'), button[type='submit'], button.btn-save").first to be visible </t>
+          <t>2026-08-29 21:05:12</t>
         </is>
       </c>
     </row>
@@ -12421,7 +12461,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J6" s="0" t="inlineStr">
@@ -12431,7 +12471,7 @@
       </c>
       <c r="K6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-29 20:24:21 | Locator.wait_for: Timeout 8000ms exceeded. Call log:   - waiting for locator("button:has-text('Save'), button:has-text('Submit'), button[type='submit'], button.btn-save").first to be visible </t>
+          <t>2026-08-29 21:05:26</t>
         </is>
       </c>
     </row>
@@ -12484,7 +12524,7 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J7" s="0" t="inlineStr">
@@ -12494,7 +12534,7 @@
       </c>
       <c r="K7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-29 20:25:27 | Locator.wait_for: Timeout 8000ms exceeded. Call log:   - waiting for locator("button:has-text('Save'), button:has-text('Submit'), button[type='submit'], button.btn-save").first to be visible </t>
+          <t>2026-08-29 21:05:38</t>
         </is>
       </c>
     </row>
@@ -12552,7 +12592,7 @@
       </c>
       <c r="K8" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 20:25:28</t>
+          <t>2026-08-29 21:05:40</t>
         </is>
       </c>
     </row>
@@ -12604,7 +12644,7 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J9" s="0" t="inlineStr">
@@ -12614,7 +12654,7 @@
       </c>
       <c r="K9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-29 20:26:37 | Locator.wait_for: Timeout 8000ms exceeded. Call log:   - waiting for locator("button:has-text('Save'), button:has-text('Submit'), button[type='submit'], button.btn-save").first to be visible </t>
+          <t>2026-08-29 21:05:53</t>
         </is>
       </c>
     </row>
@@ -12669,7 +12709,7 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J10" s="0" t="inlineStr">
@@ -12679,7 +12719,7 @@
       </c>
       <c r="K10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-29 20:27:51 | Locator.wait_for: Timeout 8000ms exceeded. Call log:   - waiting for locator("button:has-text('Save'), button:has-text('Submit'), button[type='submit'], button.btn-save").first to be visible </t>
+          <t>2026-08-29 21:06:06</t>
         </is>
       </c>
     </row>
@@ -12734,7 +12774,7 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J11" s="0" t="inlineStr">
@@ -12744,7 +12784,7 @@
       </c>
       <c r="K11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-29 20:29:09 | Locator.wait_for: Timeout 8000ms exceeded. Call log:   - waiting for locator("button:has-text('Save'), button:has-text('Submit'), button[type='submit'], button.btn-save").first to be visible </t>
+          <t>2026-08-29 21:06:19</t>
         </is>
       </c>
     </row>
@@ -12796,7 +12836,7 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J12" s="0" t="inlineStr">
@@ -12806,7 +12846,7 @@
       </c>
       <c r="K12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-29 20:29:43 | Locator.wait_for: Timeout 8000ms exceeded. Call log:   - waiting for locator("button:has-text('Save'), button:has-text('Submit'), button[type='submit'], button.btn-save").first to be visible </t>
+          <t>2026-08-29 21:06:23</t>
         </is>
       </c>
     </row>
@@ -12858,7 +12898,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J13" s="0" t="inlineStr">
@@ -12868,7 +12908,7 @@
       </c>
       <c r="K13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-29 20:30:49 | Locator.wait_for: Timeout 8000ms exceeded. Call log:   - waiting for locator("button:has-text('Save'), button:has-text('Submit'), button[type='submit'], button.btn-save").first to be visible </t>
+          <t>2026-08-29 21:06:29</t>
         </is>
       </c>
     </row>
@@ -12921,7 +12961,7 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J14" s="0" t="inlineStr">
@@ -12931,7 +12971,7 @@
       </c>
       <c r="K14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-29 20:32:00 | Locator.wait_for: Timeout 8000ms exceeded. Call log:   - waiting for locator("button:has-text('Save'), button:has-text('Submit'), button[type='submit'], button.btn-save").first to be visible </t>
+          <t>2026-08-29 21:06:42</t>
         </is>
       </c>
     </row>
@@ -12984,7 +13024,7 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J15" s="0" t="inlineStr">
@@ -12994,7 +13034,7 @@
       </c>
       <c r="K15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-29 20:33:06 | Locator.wait_for: Timeout 8000ms exceeded. Call log:   - waiting for locator("button:has-text('Save'), button:has-text('Submit'), button[type='submit'], button.btn-save").first to be visible </t>
+          <t>2026-08-29 21:06:55</t>
         </is>
       </c>
     </row>
@@ -13046,7 +13086,7 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J16" s="0" t="inlineStr">
@@ -13056,7 +13096,7 @@
       </c>
       <c r="K16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-29 20:34:15 | Locator.wait_for: Timeout 8000ms exceeded. Call log:   - waiting for locator("button:has-text('Save'), button:has-text('Submit'), button[type='submit'], button.btn-save").first to be visible </t>
+          <t>2026-08-29 21:07:07</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(vendor): update excel test execution results
</commit_message>
<xml_diff>
--- a/swarajya-create/vendor-management/test_data/Create-Vendor-Management.xlsx
+++ b/swarajya-create/vendor-management/test_data/Create-Vendor-Management.xlsx
@@ -607,7 +607,7 @@
       </c>
       <c r="K2" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 21:02:58</t>
+          <t>2026-08-29 21:12:18</t>
         </is>
       </c>
     </row>
@@ -670,7 +670,7 @@
       </c>
       <c r="K3" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 21:03:10</t>
+          <t>2026-08-29 21:12:22</t>
         </is>
       </c>
     </row>
@@ -727,7 +727,7 @@
       </c>
       <c r="K4" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 21:03:18</t>
+          <t>2026-08-29 21:12:30</t>
         </is>
       </c>
     </row>
@@ -791,7 +791,7 @@
       </c>
       <c r="K5" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 21:03:22</t>
+          <t>2026-08-29 21:12:34</t>
         </is>
       </c>
     </row>
@@ -852,7 +852,7 @@
       </c>
       <c r="K6" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 21:03:33</t>
+          <t>2026-08-29 21:12:44</t>
         </is>
       </c>
     </row>
@@ -917,7 +917,7 @@
       </c>
       <c r="K7" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 21:03:44</t>
+          <t>2026-08-29 21:12:47</t>
         </is>
       </c>
     </row>
@@ -978,7 +978,7 @@
       </c>
       <c r="K8" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 21:03:49</t>
+          <t>2026-08-29 21:12:51</t>
         </is>
       </c>
     </row>
@@ -1041,7 +1041,7 @@
       </c>
       <c r="K9" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 21:03:59</t>
+          <t>2026-08-29 21:12:54</t>
         </is>
       </c>
     </row>
@@ -1104,7 +1104,7 @@
       </c>
       <c r="K10" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 21:04:10</t>
+          <t>2026-08-29 21:12:58</t>
         </is>
       </c>
     </row>
@@ -12224,7 +12224,7 @@
       </c>
       <c r="K2" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 21:04:34</t>
+          <t>2026-08-29 21:11:16</t>
         </is>
       </c>
     </row>
@@ -12286,7 +12286,7 @@
       </c>
       <c r="K3" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 21:04:47</t>
+          <t>2026-08-29 21:11:21</t>
         </is>
       </c>
     </row>
@@ -12348,7 +12348,7 @@
       </c>
       <c r="K4" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 21:05:00</t>
+          <t>2026-08-29 21:11:25</t>
         </is>
       </c>
     </row>
@@ -12408,7 +12408,7 @@
       </c>
       <c r="K5" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 21:05:12</t>
+          <t>2026-08-29 21:11:28</t>
         </is>
       </c>
     </row>
@@ -12471,7 +12471,7 @@
       </c>
       <c r="K6" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 21:05:26</t>
+          <t>2026-08-29 21:11:32</t>
         </is>
       </c>
     </row>
@@ -12534,7 +12534,7 @@
       </c>
       <c r="K7" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 21:05:38</t>
+          <t>2026-08-29 21:11:35</t>
         </is>
       </c>
     </row>
@@ -12592,7 +12592,7 @@
       </c>
       <c r="K8" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 21:05:40</t>
+          <t>2026-08-29 21:11:38</t>
         </is>
       </c>
     </row>
@@ -12654,7 +12654,7 @@
       </c>
       <c r="K9" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 21:05:53</t>
+          <t>2026-08-29 21:11:42</t>
         </is>
       </c>
     </row>
@@ -12719,7 +12719,7 @@
       </c>
       <c r="K10" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 21:06:06</t>
+          <t>2026-08-29 21:11:47</t>
         </is>
       </c>
     </row>
@@ -12784,7 +12784,7 @@
       </c>
       <c r="K11" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 21:06:19</t>
+          <t>2026-08-29 21:11:51</t>
         </is>
       </c>
     </row>
@@ -12846,7 +12846,7 @@
       </c>
       <c r="K12" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 21:06:23</t>
+          <t>2026-08-29 21:11:54</t>
         </is>
       </c>
     </row>
@@ -12908,7 +12908,7 @@
       </c>
       <c r="K13" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 21:06:29</t>
+          <t>2026-08-29 21:12:00</t>
         </is>
       </c>
     </row>
@@ -12971,7 +12971,7 @@
       </c>
       <c r="K14" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 21:06:42</t>
+          <t>2026-08-29 21:12:06</t>
         </is>
       </c>
     </row>
@@ -13034,7 +13034,7 @@
       </c>
       <c r="K15" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 21:06:55</t>
+          <t>2026-08-29 21:12:11</t>
         </is>
       </c>
     </row>
@@ -13096,7 +13096,7 @@
       </c>
       <c r="K16" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 21:07:07</t>
+          <t>2026-08-29 21:12:15</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(vendor): enforce strict positive assertions, mandatory field filling, and confirmation popup handling
</commit_message>
<xml_diff>
--- a/swarajya-create/vendor-management/test_data/Create-Vendor-Management.xlsx
+++ b/swarajya-create/vendor-management/test_data/Create-Vendor-Management.xlsx
@@ -607,7 +607,7 @@
       </c>
       <c r="K2" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 21:12:18</t>
+          <t>2026-08-30 09:06:03</t>
         </is>
       </c>
     </row>
@@ -670,7 +670,7 @@
       </c>
       <c r="K3" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 21:12:22</t>
+          <t>2026-08-30 09:06:09</t>
         </is>
       </c>
     </row>
@@ -727,7 +727,7 @@
       </c>
       <c r="K4" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 21:12:30</t>
+          <t>2026-08-30 09:06:14</t>
         </is>
       </c>
     </row>
@@ -791,7 +791,7 @@
       </c>
       <c r="K5" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 21:12:34</t>
+          <t>2026-08-30 09:06:17</t>
         </is>
       </c>
     </row>
@@ -852,7 +852,7 @@
       </c>
       <c r="K6" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 21:12:44</t>
+          <t>2026-08-30 09:06:23</t>
         </is>
       </c>
     </row>
@@ -917,7 +917,7 @@
       </c>
       <c r="K7" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 21:12:47</t>
+          <t>2026-08-30 09:06:32</t>
         </is>
       </c>
     </row>
@@ -978,7 +978,7 @@
       </c>
       <c r="K8" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 21:12:51</t>
+          <t>2026-08-30 09:06:36</t>
         </is>
       </c>
     </row>
@@ -1041,7 +1041,7 @@
       </c>
       <c r="K9" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 21:12:54</t>
+          <t>2026-08-30 09:06:45</t>
         </is>
       </c>
     </row>
@@ -1104,7 +1104,7 @@
       </c>
       <c r="K10" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 21:12:58</t>
+          <t>2026-08-30 09:06:53</t>
         </is>
       </c>
     </row>
@@ -12224,7 +12224,7 @@
       </c>
       <c r="K2" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 21:11:16</t>
+          <t>2026-08-30 09:28:20</t>
         </is>
       </c>
     </row>
@@ -12286,7 +12286,7 @@
       </c>
       <c r="K3" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 21:11:21</t>
+          <t>2026-08-30 09:28:32</t>
         </is>
       </c>
     </row>
@@ -12348,7 +12348,7 @@
       </c>
       <c r="K4" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 21:11:25</t>
+          <t>2026-08-30 09:28:43</t>
         </is>
       </c>
     </row>
@@ -12408,7 +12408,7 @@
       </c>
       <c r="K5" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 21:11:28</t>
+          <t>2026-08-30 09:28:54</t>
         </is>
       </c>
     </row>
@@ -12471,7 +12471,7 @@
       </c>
       <c r="K6" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 21:11:32</t>
+          <t>2026-08-30 09:29:05</t>
         </is>
       </c>
     </row>
@@ -12534,7 +12534,7 @@
       </c>
       <c r="K7" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 21:11:35</t>
+          <t>2026-08-30 09:29:15</t>
         </is>
       </c>
     </row>
@@ -12592,7 +12592,7 @@
       </c>
       <c r="K8" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 21:11:38</t>
+          <t>2026-08-30 09:29:17</t>
         </is>
       </c>
     </row>
@@ -12654,7 +12654,7 @@
       </c>
       <c r="K9" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 21:11:42</t>
+          <t>2026-08-30 09:29:30</t>
         </is>
       </c>
     </row>
@@ -12719,7 +12719,7 @@
       </c>
       <c r="K10" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 21:11:47</t>
+          <t>2026-08-30 09:29:41</t>
         </is>
       </c>
     </row>
@@ -12784,7 +12784,7 @@
       </c>
       <c r="K11" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 21:11:51</t>
+          <t>2026-08-30 09:29:53</t>
         </is>
       </c>
     </row>
@@ -12846,7 +12846,7 @@
       </c>
       <c r="K12" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 21:11:54</t>
+          <t>2026-08-30 09:29:57</t>
         </is>
       </c>
     </row>
@@ -12908,7 +12908,7 @@
       </c>
       <c r="K13" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 21:12:00</t>
+          <t>2026-08-30 09:30:03</t>
         </is>
       </c>
     </row>
@@ -12971,7 +12971,7 @@
       </c>
       <c r="K14" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 21:12:06</t>
+          <t>2026-08-30 09:30:18</t>
         </is>
       </c>
     </row>
@@ -13034,7 +13034,7 @@
       </c>
       <c r="K15" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 21:12:11</t>
+          <t>2026-08-30 09:30:29</t>
         </is>
       </c>
     </row>
@@ -13096,7 +13096,7 @@
       </c>
       <c r="K16" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 21:12:15</t>
+          <t>2026-08-30 09:30:45</t>
         </is>
       </c>
     </row>

</xml_diff>